<commit_message>
Backup DB / Cambios nombres Recaudación
</commit_message>
<xml_diff>
--- a/upload/productos.xlsx
+++ b/upload/productos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Educación\Python\Proyecto - Sistema de Pedidos por WhatsApp\sistema_pedidos\upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\flori\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509CC107-2F79-48FA-9252-CD14AD4348CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9E66FD-325F-43D3-8B5D-4FF995BBC3A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="259">
   <si>
     <t xml:space="preserve">Productos </t>
   </si>
@@ -54,9 +54,6 @@
     <t>hude</t>
   </si>
   <si>
-    <t>normal</t>
-  </si>
-  <si>
     <t>pisos delicados</t>
   </si>
   <si>
@@ -111,9 +108,6 @@
     <t>dest</t>
   </si>
   <si>
-    <t>1.5Lt</t>
-  </si>
-  <si>
     <t xml:space="preserve">suavitel </t>
   </si>
   <si>
@@ -129,9 +123,6 @@
     <t>400 ml</t>
   </si>
   <si>
-    <t xml:space="preserve">tiras x 12 </t>
-  </si>
-  <si>
     <t>80 ml</t>
   </si>
   <si>
@@ -141,9 +132,6 @@
     <t>ayudin</t>
   </si>
   <si>
-    <t>380 ml</t>
-  </si>
-  <si>
     <t xml:space="preserve">ayudin </t>
   </si>
   <si>
@@ -153,9 +141,6 @@
     <t>750g</t>
   </si>
   <si>
-    <t>1200g</t>
-  </si>
-  <si>
     <t xml:space="preserve">lejia </t>
   </si>
   <si>
@@ -165,9 +150,6 @@
     <t>blanco</t>
   </si>
   <si>
-    <t>4.8 L</t>
-  </si>
-  <si>
     <t xml:space="preserve">clorandina </t>
   </si>
   <si>
@@ -204,9 +186,6 @@
     <t xml:space="preserve">industrial </t>
   </si>
   <si>
-    <t>1 Lt</t>
-  </si>
-  <si>
     <t>pastilla tanque azul</t>
   </si>
   <si>
@@ -225,9 +204,6 @@
     <t>x2</t>
   </si>
   <si>
-    <t xml:space="preserve">und </t>
-  </si>
-  <si>
     <t>x3</t>
   </si>
   <si>
@@ -246,12 +222,6 @@
     <t>kreso</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>3l</t>
-  </si>
-  <si>
     <t xml:space="preserve">desatorador </t>
   </si>
   <si>
@@ -297,9 +267,6 @@
     <t>varios</t>
   </si>
   <si>
-    <t xml:space="preserve">1lt </t>
-  </si>
-  <si>
     <t>Ña Pancha</t>
   </si>
   <si>
@@ -309,9 +276,6 @@
     <t>Daryza</t>
   </si>
   <si>
-    <t>1 LT</t>
-  </si>
-  <si>
     <t>650ml</t>
   </si>
   <si>
@@ -363,12 +327,6 @@
     <t>paracas</t>
   </si>
   <si>
-    <t>negro</t>
-  </si>
-  <si>
-    <t>x4</t>
-  </si>
-  <si>
     <t xml:space="preserve">papel toalla </t>
   </si>
   <si>
@@ -685,13 +643,172 @@
   </si>
   <si>
     <t>076</t>
+  </si>
+  <si>
+    <t>trapos y trapeadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trapeador </t>
+  </si>
+  <si>
+    <t xml:space="preserve">plomo yute </t>
+  </si>
+  <si>
+    <t>fibra peluche</t>
+  </si>
+  <si>
+    <t>fibra liso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trapos </t>
+  </si>
+  <si>
+    <t>individual</t>
+  </si>
+  <si>
+    <t>trapos x4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bolsas </t>
+  </si>
+  <si>
+    <t xml:space="preserve">50 litros </t>
+  </si>
+  <si>
+    <t>46x68 cm</t>
+  </si>
+  <si>
+    <t>75 litros</t>
+  </si>
+  <si>
+    <t>65x100 cm</t>
+  </si>
+  <si>
+    <t>077</t>
+  </si>
+  <si>
+    <t>078</t>
+  </si>
+  <si>
+    <t>079</t>
+  </si>
+  <si>
+    <t>080</t>
+  </si>
+  <si>
+    <t>081</t>
+  </si>
+  <si>
+    <t>082</t>
+  </si>
+  <si>
+    <t>083</t>
+  </si>
+  <si>
+    <t>084</t>
+  </si>
+  <si>
+    <t>085</t>
+  </si>
+  <si>
+    <t>negro x4</t>
+  </si>
+  <si>
+    <t>plancha</t>
+  </si>
+  <si>
+    <t>unidad</t>
+  </si>
+  <si>
+    <t>086</t>
+  </si>
+  <si>
+    <t>escobon</t>
+  </si>
+  <si>
+    <t>clasico</t>
+  </si>
+  <si>
+    <t>280 ml</t>
+  </si>
+  <si>
+    <t>4.7L</t>
+  </si>
+  <si>
+    <t>3.8 L</t>
+  </si>
+  <si>
+    <t>color</t>
+  </si>
+  <si>
+    <t>galon</t>
+  </si>
+  <si>
+    <t>1 L</t>
+  </si>
+  <si>
+    <t>1l</t>
+  </si>
+  <si>
+    <t>1gll</t>
+  </si>
+  <si>
+    <t>1.5L</t>
+  </si>
+  <si>
+    <t>repuesto x3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">secador </t>
+  </si>
+  <si>
+    <t>secador</t>
+  </si>
+  <si>
+    <t>aromatisante</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>30 gr</t>
+  </si>
+  <si>
+    <t>087</t>
+  </si>
+  <si>
+    <t>088</t>
+  </si>
+  <si>
+    <t>300ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">900gr </t>
+  </si>
+  <si>
+    <t>escobilla</t>
+  </si>
+  <si>
+    <t>HUDE</t>
+  </si>
+  <si>
+    <t>089</t>
+  </si>
+  <si>
+    <t>090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psata </t>
+  </si>
+  <si>
+    <t>1.100g</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -736,8 +853,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -852,8 +975,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -928,8 +1057,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="20">
+  <cellStyleXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
@@ -950,8 +1097,9 @@
     <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="11" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="4" xfId="11" applyBorder="1" applyAlignment="1">
@@ -1105,6 +1253,50 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="20" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="20" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="20" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="8" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="20" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="20" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="7" xfId="20" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="5" xfId="20" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="21" borderId="4" xfId="20" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="6" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="13" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="5" xfId="13" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="3" xfId="13" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1121,15 +1313,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="2" xfId="13" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="5" xfId="13" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="3" xfId="13" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="7" applyBorder="1" applyAlignment="1">
@@ -1226,7 +1409,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="20">
+  <cellStyles count="21">
     <cellStyle name="20% - Énfasis1" xfId="3" builtinId="30"/>
     <cellStyle name="20% - Énfasis2" xfId="5" builtinId="34"/>
     <cellStyle name="20% - Énfasis4" xfId="11" builtinId="42"/>
@@ -1234,6 +1417,7 @@
     <cellStyle name="20% - Énfasis6" xfId="18" builtinId="50"/>
     <cellStyle name="40% - Énfasis1" xfId="4" builtinId="31"/>
     <cellStyle name="40% - Énfasis2" xfId="6" builtinId="35"/>
+    <cellStyle name="40% - Énfasis3" xfId="20" builtinId="39"/>
     <cellStyle name="40% - Énfasis4" xfId="12" builtinId="43"/>
     <cellStyle name="60% - Énfasis2" xfId="7" builtinId="36"/>
     <cellStyle name="60% - Énfasis3" xfId="9" builtinId="40"/>
@@ -1524,7 +1708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:H81"/>
+  <dimension ref="B3:H95"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9.140625" style="64"/>
@@ -1534,52 +1718,55 @@
     <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="65" t="s">
-        <v>142</v>
-      </c>
-      <c r="C3" s="65" t="s">
+      <c r="B3" s="83" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="65" t="s">
+      <c r="D3" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="65" t="s">
+      <c r="E3" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="65" t="s">
+      <c r="F3" s="83" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="103" t="s">
+      <c r="G3" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="65" t="s">
+      <c r="H3" s="83" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="104"/>
-      <c r="H4" s="66"/>
+      <c r="B4" s="84"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="119"/>
+      <c r="H4" s="84"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C5" s="77" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" s="92" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+      <c r="F5" s="1" t="s">
+        <v>233</v>
+      </c>
       <c r="G5" s="2">
         <v>1</v>
       </c>
@@ -1589,15 +1776,15 @@
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C6" s="102"/>
+        <v>130</v>
+      </c>
+      <c r="C6" s="117"/>
       <c r="D6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>232</v>
       </c>
       <c r="G6" s="4">
         <v>2</v>
@@ -1608,15 +1795,15 @@
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="C7" s="78"/>
+        <v>131</v>
+      </c>
+      <c r="C7" s="93"/>
       <c r="D7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G7" s="5">
         <v>3</v>
@@ -1627,10 +1814,10 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>8</v>
@@ -1646,17 +1833,17 @@
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="C9" s="99" t="s">
+        <v>133</v>
+      </c>
+      <c r="C9" s="114" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>13</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>14</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G9" s="10">
         <v>4</v>
@@ -1667,15 +1854,15 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C10" s="100"/>
+        <v>134</v>
+      </c>
+      <c r="C10" s="115"/>
       <c r="D10" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G10" s="10">
         <v>3</v>
@@ -1686,15 +1873,15 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C11" s="100"/>
+        <v>135</v>
+      </c>
+      <c r="C11" s="115"/>
       <c r="D11" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11" s="10">
         <v>2</v>
@@ -1705,15 +1892,15 @@
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="100"/>
+        <v>136</v>
+      </c>
+      <c r="C12" s="115"/>
       <c r="D12" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G12" s="10">
         <v>1</v>
@@ -1724,15 +1911,15 @@
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="100"/>
+        <v>137</v>
+      </c>
+      <c r="C13" s="115"/>
       <c r="D13" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G13" s="10">
         <v>9</v>
@@ -1743,15 +1930,15 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="C14" s="100"/>
+        <v>138</v>
+      </c>
+      <c r="C14" s="115"/>
       <c r="D14" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G14" s="10">
         <v>10</v>
@@ -1762,15 +1949,15 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="C15" s="100"/>
+        <v>139</v>
+      </c>
+      <c r="C15" s="115"/>
       <c r="D15" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G15" s="10">
         <v>4</v>
@@ -1781,15 +1968,15 @@
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="C16" s="100"/>
+        <v>140</v>
+      </c>
+      <c r="C16" s="115"/>
       <c r="D16" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G16" s="10">
         <v>4</v>
@@ -1800,12 +1987,12 @@
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C17" s="100"/>
+        <v>141</v>
+      </c>
+      <c r="C17" s="115"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="10">
@@ -1815,17 +2002,17 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C18" s="101"/>
+        <v>142</v>
+      </c>
+      <c r="C18" s="116"/>
       <c r="D18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>25</v>
       </c>
       <c r="G18" s="10">
         <v>12</v>
@@ -1834,19 +2021,19 @@
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="C19" s="87" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="102" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="12" t="s">
-        <v>27</v>
-      </c>
       <c r="E19" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>28</v>
+        <v>242</v>
       </c>
       <c r="G19" s="13">
         <v>6</v>
@@ -1857,15 +2044,15 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="C20" s="88"/>
+        <v>144</v>
+      </c>
+      <c r="C20" s="103"/>
       <c r="D20" s="12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E20" s="12"/>
       <c r="F20" s="12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G20" s="13">
         <v>6</v>
@@ -1876,15 +2063,15 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="C21" s="88"/>
+        <v>145</v>
+      </c>
+      <c r="C21" s="103"/>
       <c r="D21" s="12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G21" s="13">
         <v>12</v>
@@ -1895,15 +2082,15 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="C22" s="88"/>
+        <v>146</v>
+      </c>
+      <c r="C22" s="103"/>
       <c r="D22" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E22" s="12"/>
       <c r="F22" s="12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G22" s="13">
         <v>12</v>
@@ -1914,15 +2101,15 @@
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="C23" s="88"/>
+        <v>147</v>
+      </c>
+      <c r="C23" s="103"/>
       <c r="D23" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E23" s="12"/>
       <c r="F23" s="12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G23" s="13">
         <v>6</v>
@@ -1933,32 +2120,30 @@
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="C24" s="88"/>
+        <v>148</v>
+      </c>
+      <c r="C24" s="103"/>
       <c r="D24" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>34</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E24" s="12"/>
       <c r="F24" s="12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G24" s="13">
         <v>12</v>
       </c>
       <c r="H24" s="14">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="C25" s="89"/>
+        <v>149</v>
+      </c>
+      <c r="C25" s="104"/>
       <c r="D25" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E25" s="12"/>
       <c r="F25" s="12">
@@ -1971,19 +2156,19 @@
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="15" t="s">
-        <v>164</v>
-      </c>
-      <c r="C26" s="82" t="s">
-        <v>36</v>
+        <v>150</v>
+      </c>
+      <c r="C26" s="97" t="s">
+        <v>33</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>38</v>
+        <v>234</v>
       </c>
       <c r="G26" s="16">
         <v>12</v>
@@ -1994,17 +2179,17 @@
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="15" t="s">
-        <v>165</v>
-      </c>
-      <c r="C27" s="83"/>
+        <v>151</v>
+      </c>
+      <c r="C27" s="98"/>
       <c r="D27" s="15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G27" s="16">
         <v>12</v>
@@ -2015,13 +2200,17 @@
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="C28" s="84"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
+        <v>152</v>
+      </c>
+      <c r="C28" s="99"/>
+      <c r="D28" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>257</v>
+      </c>
       <c r="F28" s="15" t="s">
-        <v>42</v>
+        <v>258</v>
       </c>
       <c r="G28" s="16">
         <v>0</v>
@@ -2030,19 +2219,19 @@
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="C29" s="96" t="s">
-        <v>43</v>
+        <v>153</v>
+      </c>
+      <c r="C29" s="111" t="s">
+        <v>38</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F29" s="18" t="s">
-        <v>46</v>
+        <v>235</v>
       </c>
       <c r="G29" s="19">
         <v>8</v>
@@ -2053,17 +2242,17 @@
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="C30" s="97"/>
+        <v>154</v>
+      </c>
+      <c r="C30" s="112"/>
       <c r="D30" s="18" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="18">
-        <v>3.8</v>
+        <v>40</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>236</v>
       </c>
       <c r="G30" s="19">
         <v>4</v>
@@ -2074,17 +2263,17 @@
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="C31" s="97"/>
+        <v>155</v>
+      </c>
+      <c r="C31" s="112"/>
       <c r="D31" s="18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F31" s="18" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G31" s="19">
         <v>6</v>
@@ -2095,17 +2284,17 @@
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="C32" s="97"/>
+        <v>156</v>
+      </c>
+      <c r="C32" s="112"/>
       <c r="D32" s="18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F32" s="18" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="G32" s="19">
         <v>18</v>
@@ -2116,17 +2305,17 @@
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="C33" s="97"/>
+        <v>157</v>
+      </c>
+      <c r="C33" s="112"/>
       <c r="D33" s="18" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="F33" s="18" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G33" s="19">
         <v>15</v>
@@ -2137,16 +2326,18 @@
     </row>
     <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="C34" s="97"/>
+        <v>158</v>
+      </c>
+      <c r="C34" s="112"/>
       <c r="D34" s="18" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F34" s="18"/>
+        <v>47</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>237</v>
+      </c>
       <c r="G34" s="19">
         <v>4</v>
       </c>
@@ -2156,16 +2347,18 @@
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="C35" s="97"/>
+        <v>159</v>
+      </c>
+      <c r="C35" s="112"/>
       <c r="D35" s="18" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F35" s="18"/>
+        <v>47</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>47</v>
+      </c>
       <c r="G35" s="19">
         <v>4</v>
       </c>
@@ -2175,16 +2368,18 @@
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" s="18" t="s">
-        <v>174</v>
-      </c>
-      <c r="C36" s="98"/>
+        <v>160</v>
+      </c>
+      <c r="C36" s="113"/>
       <c r="D36" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="E36" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="18"/>
+      <c r="F36" s="18" t="s">
+        <v>47</v>
+      </c>
       <c r="G36" s="19">
         <v>2</v>
       </c>
@@ -2194,17 +2389,17 @@
     </row>
     <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" s="21" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E37" s="21"/>
       <c r="F37" s="21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G37" s="22">
         <v>12</v>
@@ -2213,17 +2408,17 @@
     </row>
     <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" s="24" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="C38" s="24" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D38" s="24" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E38" s="24"/>
       <c r="F38" s="24" t="s">
-        <v>59</v>
+        <v>239</v>
       </c>
       <c r="G38" s="25">
         <v>12</v>
@@ -2234,19 +2429,19 @@
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" s="27" t="s">
-        <v>177</v>
-      </c>
-      <c r="C39" s="93" t="s">
-        <v>60</v>
+        <v>163</v>
+      </c>
+      <c r="C39" s="108" t="s">
+        <v>53</v>
       </c>
       <c r="D39" s="27" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E39" s="27" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="G39" s="28">
         <v>24</v>
@@ -2257,17 +2452,17 @@
     </row>
     <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="C40" s="94"/>
+        <v>164</v>
+      </c>
+      <c r="C40" s="109"/>
       <c r="D40" s="27" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E40" s="27" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="G40" s="28">
         <v>24</v>
@@ -2278,15 +2473,15 @@
     </row>
     <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" s="27" t="s">
-        <v>179</v>
-      </c>
-      <c r="C41" s="95"/>
+        <v>165</v>
+      </c>
+      <c r="C41" s="110"/>
       <c r="D41" s="27"/>
       <c r="E41" s="27" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F41" s="27" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="G41" s="28">
         <v>0</v>
@@ -2295,17 +2490,17 @@
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" s="30" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D42" s="30" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="E42" s="30"/>
       <c r="F42" s="30" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G42" s="31">
         <v>24</v>
@@ -2316,17 +2511,17 @@
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="33" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D43" s="33" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E43" s="33"/>
       <c r="F43" s="33" t="s">
-        <v>74</v>
+        <v>238</v>
       </c>
       <c r="G43" s="34">
         <v>6</v>
@@ -2337,19 +2532,19 @@
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="36" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="C44" s="36" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D44" s="36" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E44" s="36" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F44" s="36" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="G44" s="37">
         <v>12</v>
@@ -2358,19 +2553,19 @@
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="39" t="s">
-        <v>183</v>
-      </c>
-      <c r="C45" s="74" t="s">
-        <v>79</v>
+        <v>169</v>
+      </c>
+      <c r="C45" s="89" t="s">
+        <v>69</v>
       </c>
       <c r="D45" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="E45" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="E45" s="39" t="s">
-        <v>80</v>
-      </c>
       <c r="F45" s="39" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="G45" s="40">
         <v>8</v>
@@ -2381,15 +2576,17 @@
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="C46" s="75"/>
-      <c r="D46" s="39"/>
+        <v>170</v>
+      </c>
+      <c r="C46" s="90"/>
+      <c r="D46" s="39" t="s">
+        <v>62</v>
+      </c>
       <c r="E46" s="39" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="F46" s="39" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="G46" s="40">
         <v>8</v>
@@ -2400,15 +2597,17 @@
     </row>
     <row r="47" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B47" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="C47" s="76"/>
-      <c r="D47" s="39"/>
+        <v>171</v>
+      </c>
+      <c r="C47" s="91"/>
+      <c r="D47" s="39" t="s">
+        <v>62</v>
+      </c>
       <c r="E47" s="39" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="F47" s="39" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="G47" s="40">
         <v>8</v>
@@ -2419,17 +2618,17 @@
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B48" s="42" t="s">
-        <v>186</v>
-      </c>
-      <c r="C48" s="85" t="s">
-        <v>83</v>
+        <v>172</v>
+      </c>
+      <c r="C48" s="100" t="s">
+        <v>73</v>
       </c>
       <c r="D48" s="42" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E48" s="42"/>
       <c r="F48" s="42" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G48" s="43">
         <v>12</v>
@@ -2440,15 +2639,15 @@
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B49" s="42" t="s">
-        <v>187</v>
-      </c>
-      <c r="C49" s="86"/>
+        <v>173</v>
+      </c>
+      <c r="C49" s="101"/>
       <c r="D49" s="42" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="E49" s="42"/>
       <c r="F49" s="42" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G49" s="43">
         <v>12</v>
@@ -2459,19 +2658,19 @@
     </row>
     <row r="50" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B50" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="C50" s="87" t="s">
-        <v>87</v>
+        <v>174</v>
+      </c>
+      <c r="C50" s="102" t="s">
+        <v>77</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="G50" s="13">
         <v>12</v>
@@ -2482,17 +2681,17 @@
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B51" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="C51" s="88"/>
+        <v>175</v>
+      </c>
+      <c r="C51" s="103"/>
       <c r="D51" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F51" s="12" t="s">
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="G51" s="13">
         <v>24</v>
@@ -2503,17 +2702,17 @@
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B52" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="C52" s="89"/>
+        <v>176</v>
+      </c>
+      <c r="C52" s="104"/>
       <c r="D52" s="12" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>25</v>
+        <v>241</v>
       </c>
       <c r="G52" s="13">
         <v>24</v>
@@ -2524,17 +2723,17 @@
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B53" s="45" t="s">
-        <v>191</v>
-      </c>
-      <c r="C53" s="90" t="s">
-        <v>92</v>
+        <v>177</v>
+      </c>
+      <c r="C53" s="105" t="s">
+        <v>81</v>
       </c>
       <c r="D53" s="45" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="E53" s="45"/>
       <c r="F53" s="45" t="s">
-        <v>94</v>
+        <v>239</v>
       </c>
       <c r="G53" s="46">
         <v>6</v>
@@ -2545,15 +2744,15 @@
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B54" s="45" t="s">
-        <v>192</v>
-      </c>
-      <c r="C54" s="91"/>
+        <v>178</v>
+      </c>
+      <c r="C54" s="106"/>
       <c r="D54" s="45" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E54" s="45"/>
       <c r="F54" s="45" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="G54" s="46">
         <v>6</v>
@@ -2563,20 +2762,20 @@
       </c>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B55" s="67" t="s">
-        <v>193</v>
-      </c>
-      <c r="C55" s="67" t="s">
-        <v>96</v>
-      </c>
-      <c r="D55" s="67" t="s">
-        <v>97</v>
+      <c r="B55" s="85" t="s">
+        <v>179</v>
+      </c>
+      <c r="C55" s="85" t="s">
+        <v>84</v>
+      </c>
+      <c r="D55" s="85" t="s">
+        <v>85</v>
       </c>
       <c r="E55" s="24" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F55" s="24" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G55" s="25">
         <v>12</v>
@@ -2586,16 +2785,16 @@
       </c>
     </row>
     <row r="56" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B56" s="68" t="s">
-        <v>194</v>
-      </c>
-      <c r="C56" s="68"/>
-      <c r="D56" s="68"/>
+      <c r="B56" s="86" t="s">
+        <v>180</v>
+      </c>
+      <c r="C56" s="86"/>
+      <c r="D56" s="86"/>
       <c r="E56" s="24" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F56" s="24" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="G56" s="25">
         <v>12</v>
@@ -2605,16 +2804,16 @@
       </c>
     </row>
     <row r="57" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B57" s="68" t="s">
-        <v>195</v>
-      </c>
-      <c r="C57" s="68"/>
-      <c r="D57" s="68"/>
+      <c r="B57" s="86" t="s">
+        <v>181</v>
+      </c>
+      <c r="C57" s="86"/>
+      <c r="D57" s="86"/>
       <c r="E57" s="24" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F57" s="24" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G57" s="25">
         <v>12</v>
@@ -2624,16 +2823,16 @@
       </c>
     </row>
     <row r="58" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B58" s="68" t="s">
-        <v>196</v>
-      </c>
-      <c r="C58" s="68"/>
-      <c r="D58" s="68"/>
+      <c r="B58" s="86" t="s">
+        <v>182</v>
+      </c>
+      <c r="C58" s="86"/>
+      <c r="D58" s="86"/>
       <c r="E58" s="24" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F58" s="24" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="G58" s="25">
         <v>12</v>
@@ -2643,16 +2842,16 @@
       </c>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B59" s="68" t="s">
-        <v>197</v>
-      </c>
-      <c r="C59" s="68"/>
-      <c r="D59" s="68"/>
+      <c r="B59" s="86" t="s">
+        <v>183</v>
+      </c>
+      <c r="C59" s="86"/>
+      <c r="D59" s="86"/>
       <c r="E59" s="24" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F59" s="24" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G59" s="25">
         <v>12</v>
@@ -2662,16 +2861,16 @@
       </c>
     </row>
     <row r="60" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B60" s="68" t="s">
-        <v>198</v>
-      </c>
-      <c r="C60" s="92"/>
-      <c r="D60" s="68"/>
+      <c r="B60" s="86" t="s">
+        <v>184</v>
+      </c>
+      <c r="C60" s="107"/>
+      <c r="D60" s="86"/>
       <c r="E60" s="24" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F60" s="24" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G60" s="25">
         <v>12</v>
@@ -2682,17 +2881,17 @@
     </row>
     <row r="61" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B61" s="49" t="s">
-        <v>199</v>
-      </c>
-      <c r="C61" s="69" t="s">
-        <v>103</v>
+        <v>185</v>
+      </c>
+      <c r="C61" s="87" t="s">
+        <v>91</v>
       </c>
       <c r="D61" s="49" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E61" s="49"/>
       <c r="F61" s="49" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="G61" s="50">
         <v>6</v>
@@ -2703,15 +2902,15 @@
     </row>
     <row r="62" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B62" s="49" t="s">
-        <v>200</v>
-      </c>
-      <c r="C62" s="70"/>
+        <v>186</v>
+      </c>
+      <c r="C62" s="88"/>
       <c r="D62" s="49" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="E62" s="49"/>
       <c r="F62" s="49" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="G62" s="50">
         <v>6</v>
@@ -2722,61 +2921,61 @@
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B63" s="52" t="s">
-        <v>201</v>
-      </c>
-      <c r="C63" s="71" t="s">
-        <v>106</v>
+        <v>187</v>
+      </c>
+      <c r="C63" s="80" t="s">
+        <v>94</v>
       </c>
       <c r="D63" s="52" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="E63" s="52" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="F63" s="52" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="G63" s="53">
         <v>3</v>
       </c>
       <c r="H63" s="54">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B64" s="52" t="s">
-        <v>202</v>
-      </c>
-      <c r="C64" s="72"/>
+        <v>188</v>
+      </c>
+      <c r="C64" s="81"/>
       <c r="D64" s="52" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="E64" s="52" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="F64" s="52" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="G64" s="53">
         <v>3</v>
       </c>
       <c r="H64" s="54">
-        <v>31</v>
+        <v>21</v>
       </c>
     </row>
     <row r="65" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B65" s="52" t="s">
-        <v>203</v>
-      </c>
-      <c r="C65" s="73"/>
+        <v>189</v>
+      </c>
+      <c r="C65" s="81"/>
       <c r="D65" s="52" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E65" s="52" t="s">
-        <v>112</v>
+        <v>228</v>
       </c>
       <c r="F65" s="52" t="s">
-        <v>113</v>
+        <v>229</v>
       </c>
       <c r="G65" s="53">
         <v>24</v>
@@ -2786,323 +2985,600 @@
       </c>
     </row>
     <row r="66" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B66" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="C66" s="74" t="s">
-        <v>114</v>
-      </c>
-      <c r="D66" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="E66" s="39"/>
-      <c r="F66" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="G66" s="40">
+      <c r="B66" s="52" t="s">
+        <v>190</v>
+      </c>
+      <c r="C66" s="82"/>
+      <c r="D66" s="52" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66" s="52" t="s">
+        <v>228</v>
+      </c>
+      <c r="F66" s="52" t="s">
+        <v>230</v>
+      </c>
+      <c r="G66" s="53">
         <v>12</v>
       </c>
-      <c r="H66" s="55">
-        <v>13.5</v>
+      <c r="H66" s="54">
+        <v>7</v>
       </c>
     </row>
     <row r="67" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B67" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="C67" s="75"/>
+      <c r="B67" s="52" t="s">
+        <v>191</v>
+      </c>
+      <c r="C67" s="89" t="s">
+        <v>100</v>
+      </c>
       <c r="D67" s="39" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E67" s="39"/>
       <c r="F67" s="39" t="s">
-        <v>116</v>
+        <v>55</v>
       </c>
       <c r="G67" s="40">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H67" s="55">
-        <v>11</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="68" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B68" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="C68" s="76"/>
+      <c r="B68" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="C68" s="90"/>
       <c r="D68" s="39" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="E68" s="39"/>
       <c r="F68" s="39" t="s">
-        <v>62</v>
+        <v>102</v>
       </c>
       <c r="G68" s="40">
+        <v>18</v>
+      </c>
+      <c r="H68" s="55">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B69" s="52" t="s">
+        <v>193</v>
+      </c>
+      <c r="C69" s="91"/>
+      <c r="D69" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="E69" s="39"/>
+      <c r="F69" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="G69" s="40">
         <v>36</v>
       </c>
-      <c r="H68" s="55">
+      <c r="H69" s="55">
         <v>2.5</v>
       </c>
     </row>
-    <row r="69" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B69" s="39" t="s">
-        <v>207</v>
-      </c>
-      <c r="C69" s="56" t="s">
-        <v>118</v>
-      </c>
-      <c r="D69" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="E69" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="F69" s="39"/>
-      <c r="G69" s="40">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B70" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="C70" s="56" t="s">
+        <v>104</v>
+      </c>
+      <c r="D70" s="39" t="s">
+        <v>105</v>
+      </c>
+      <c r="E70" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="F70" s="39" t="s">
+        <v>247</v>
+      </c>
+      <c r="G70" s="40">
         <v>18</v>
       </c>
-      <c r="H69" s="55">
+      <c r="H70" s="55">
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B70" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C70" s="77" t="s">
-        <v>121</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E70" s="1"/>
-      <c r="F70" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="G70" s="2">
-        <v>12</v>
-      </c>
-      <c r="H70" s="3">
-        <v>8</v>
-      </c>
-    </row>
     <row r="71" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B71" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="C71" s="78"/>
+      <c r="B71" s="52" t="s">
+        <v>195</v>
+      </c>
+      <c r="C71" s="92" t="s">
+        <v>107</v>
+      </c>
       <c r="D71" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E71" s="1"/>
       <c r="F71" s="1" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="G71" s="2">
+        <v>12</v>
+      </c>
+      <c r="H71" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B72" s="52" t="s">
+        <v>196</v>
+      </c>
+      <c r="C72" s="93"/>
+      <c r="D72" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="G72" s="2">
         <v>6</v>
       </c>
-      <c r="H71" s="3">
+      <c r="H72" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B72" s="57" t="s">
-        <v>210</v>
-      </c>
-      <c r="C72" s="57" t="s">
-        <v>125</v>
-      </c>
-      <c r="D72" s="57" t="s">
-        <v>70</v>
-      </c>
-      <c r="E72" s="57"/>
-      <c r="F72" s="57" t="s">
-        <v>126</v>
-      </c>
-      <c r="G72" s="58">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B73" s="52" t="s">
+        <v>197</v>
+      </c>
+      <c r="C73" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="D73" s="57" t="s">
+        <v>62</v>
+      </c>
+      <c r="E73" s="57"/>
+      <c r="F73" s="57" t="s">
+        <v>112</v>
+      </c>
+      <c r="G73" s="58">
         <v>12</v>
       </c>
-      <c r="H72" s="59">
+      <c r="H73" s="59">
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B73" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="C73" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="E73" s="6"/>
-      <c r="F73" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="G73" s="7">
-        <v>48</v>
-      </c>
-      <c r="H73" s="8">
-        <v>3</v>
-      </c>
-    </row>
     <row r="74" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B74" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="C74" s="80"/>
+      <c r="B74" s="52" t="s">
+        <v>198</v>
+      </c>
+      <c r="C74" s="94" t="s">
+        <v>113</v>
+      </c>
       <c r="D74" s="6" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="G74" s="7">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="H74" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B75" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="C75" s="81"/>
+      <c r="B75" s="52" t="s">
+        <v>199</v>
+      </c>
+      <c r="C75" s="95"/>
       <c r="D75" s="6" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="E75" s="6"/>
       <c r="F75" s="6" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="G75" s="7">
         <v>20</v>
       </c>
       <c r="H75" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B76" s="52" t="s">
+        <v>200</v>
+      </c>
+      <c r="C76" s="96"/>
+      <c r="D76" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G76" s="7">
+        <v>20</v>
+      </c>
+      <c r="H76" s="8">
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B76" s="15" t="s">
-        <v>214</v>
-      </c>
-      <c r="C76" s="82" t="s">
-        <v>131</v>
-      </c>
-      <c r="D76" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="E76" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F76" s="15"/>
-      <c r="G76" s="16">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B77" s="52" t="s">
+        <v>201</v>
+      </c>
+      <c r="C77" s="97" t="s">
+        <v>117</v>
+      </c>
+      <c r="D77" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E77" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F77" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="G77" s="16">
         <v>6</v>
       </c>
-      <c r="H76" s="17">
+      <c r="H77" s="17">
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B77" s="15" t="s">
-        <v>215</v>
-      </c>
-      <c r="C77" s="83"/>
-      <c r="D77" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="E77" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="F77" s="15"/>
-      <c r="G77" s="16">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B78" s="52" t="s">
+        <v>202</v>
+      </c>
+      <c r="C78" s="98"/>
+      <c r="D78" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E78" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="G78" s="16">
         <v>15</v>
       </c>
-      <c r="H77" s="17">
+      <c r="H78" s="17">
         <v>1.5</v>
       </c>
     </row>
-    <row r="78" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B78" s="15" t="s">
-        <v>216</v>
-      </c>
-      <c r="C78" s="84"/>
-      <c r="D78" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="E78" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="F78" s="15"/>
-      <c r="G78" s="16">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B79" s="52" t="s">
+        <v>203</v>
+      </c>
+      <c r="C79" s="99"/>
+      <c r="D79" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E79" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F79" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="G79" s="16">
         <v>7</v>
       </c>
-      <c r="H78" s="17">
+      <c r="H79" s="17">
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B79" s="49" t="s">
-        <v>217</v>
-      </c>
-      <c r="C79" s="69" t="s">
-        <v>136</v>
-      </c>
-      <c r="D79" s="49" t="s">
-        <v>137</v>
-      </c>
-      <c r="E79" s="49"/>
-      <c r="F79" s="49"/>
-      <c r="G79" s="50">
-        <v>3</v>
-      </c>
-      <c r="H79" s="51">
-        <v>28</v>
-      </c>
-    </row>
     <row r="80" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B80" s="49" t="s">
-        <v>218</v>
-      </c>
-      <c r="C80" s="70"/>
+      <c r="B80" s="52" t="s">
+        <v>204</v>
+      </c>
+      <c r="C80" s="87" t="s">
+        <v>122</v>
+      </c>
       <c r="D80" s="49" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="E80" s="49"/>
-      <c r="F80" s="49"/>
+      <c r="F80" s="49" t="s">
+        <v>246</v>
+      </c>
       <c r="G80" s="50">
         <v>3</v>
       </c>
       <c r="H80" s="51">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B81" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C81" s="88"/>
+      <c r="D81" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="E81" s="49"/>
+      <c r="F81" s="49" t="s">
+        <v>243</v>
+      </c>
+      <c r="G81" s="50">
+        <v>3</v>
+      </c>
+      <c r="H81" s="51">
         <v>42</v>
       </c>
     </row>
-    <row r="81" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B81" s="60" t="s">
+    <row r="82" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B82" s="52" t="s">
         <v>219</v>
       </c>
-      <c r="C81" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="D81" s="60" t="s">
-        <v>140</v>
-      </c>
-      <c r="E81" s="60" t="s">
-        <v>141</v>
-      </c>
-      <c r="F81" s="60"/>
-      <c r="G81" s="61">
+      <c r="C82" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D82" s="60" t="s">
+        <v>126</v>
+      </c>
+      <c r="E82" s="60" t="s">
+        <v>127</v>
+      </c>
+      <c r="F82" s="60" t="s">
+        <v>248</v>
+      </c>
+      <c r="G82" s="61">
         <v>48</v>
       </c>
-      <c r="H81" s="62">
+      <c r="H82" s="62">
         <v>2.5</v>
       </c>
     </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B83" s="52" t="s">
+        <v>220</v>
+      </c>
+      <c r="C83" s="77" t="s">
+        <v>206</v>
+      </c>
+      <c r="D83" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="F83" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="G83" s="66">
+        <v>12</v>
+      </c>
+      <c r="H83" s="67">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B84" s="52" t="s">
+        <v>221</v>
+      </c>
+      <c r="C84" s="77"/>
+      <c r="D84" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="F84" s="65" t="s">
+        <v>209</v>
+      </c>
+      <c r="G84" s="66">
+        <v>12</v>
+      </c>
+      <c r="H84" s="67">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B85" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="C85" s="77"/>
+      <c r="D85" s="65" t="s">
+        <v>207</v>
+      </c>
+      <c r="F85" s="65" t="s">
+        <v>210</v>
+      </c>
+      <c r="G85" s="66">
+        <v>12</v>
+      </c>
+      <c r="H85" s="67">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B86" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="C86" s="77"/>
+      <c r="D86" s="65" t="s">
+        <v>211</v>
+      </c>
+      <c r="F86" s="65" t="s">
+        <v>212</v>
+      </c>
+      <c r="G86" s="66">
+        <v>12</v>
+      </c>
+      <c r="H86" s="67">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="87" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B87" s="52" t="s">
+        <v>224</v>
+      </c>
+      <c r="C87" s="77"/>
+      <c r="D87" s="65" t="s">
+        <v>213</v>
+      </c>
+      <c r="F87" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="G87" s="66">
+        <v>3</v>
+      </c>
+      <c r="H87" s="67">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B88" s="52" t="s">
+        <v>225</v>
+      </c>
+      <c r="C88" s="77"/>
+      <c r="D88" s="65" t="s">
+        <v>244</v>
+      </c>
+      <c r="E88" s="65"/>
+      <c r="F88" s="65" t="s">
+        <v>233</v>
+      </c>
+      <c r="G88" s="66">
+        <v>12</v>
+      </c>
+      <c r="H88" s="67">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="89" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B89" s="52" t="s">
+        <v>226</v>
+      </c>
+      <c r="C89" s="77"/>
+      <c r="D89" s="65" t="s">
+        <v>245</v>
+      </c>
+      <c r="E89" s="65"/>
+      <c r="F89" s="65" t="s">
+        <v>93</v>
+      </c>
+      <c r="G89" s="66">
+        <v>3</v>
+      </c>
+      <c r="H89" s="67">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="90" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B90" s="52" t="s">
+        <v>227</v>
+      </c>
+      <c r="C90" s="78" t="s">
+        <v>214</v>
+      </c>
+      <c r="D90" s="68" t="s">
+        <v>215</v>
+      </c>
+      <c r="F90" s="69" t="s">
+        <v>216</v>
+      </c>
+      <c r="G90" s="70">
+        <v>20</v>
+      </c>
+      <c r="H90" s="71">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B91" s="52" t="s">
+        <v>231</v>
+      </c>
+      <c r="C91" s="79"/>
+      <c r="D91" s="68" t="s">
+        <v>217</v>
+      </c>
+      <c r="F91" s="69" t="s">
+        <v>218</v>
+      </c>
+      <c r="G91" s="70">
+        <v>10</v>
+      </c>
+      <c r="H91" s="71">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B92" s="52" t="s">
+        <v>249</v>
+      </c>
+      <c r="C92" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D92" s="72" t="s">
+        <v>22</v>
+      </c>
+      <c r="F92" s="73" t="s">
+        <v>251</v>
+      </c>
+      <c r="G92" s="74">
+        <v>24</v>
+      </c>
+      <c r="H92" s="75">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="93" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B93" s="52" t="s">
+        <v>250</v>
+      </c>
+      <c r="C93" s="63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D93" s="72" t="s">
+        <v>126</v>
+      </c>
+      <c r="F93" s="73" t="s">
+        <v>252</v>
+      </c>
+      <c r="G93">
+        <v>6</v>
+      </c>
+      <c r="H93" s="75">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="94" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B94" s="52" t="s">
+        <v>255</v>
+      </c>
+      <c r="C94" s="76" t="s">
+        <v>253</v>
+      </c>
+      <c r="D94" s="72" t="s">
+        <v>254</v>
+      </c>
+      <c r="G94">
+        <v>6</v>
+      </c>
+      <c r="H94" s="75">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B95" s="52" t="s">
+        <v>256</v>
+      </c>
+      <c r="C95" s="76" t="s">
+        <v>65</v>
+      </c>
+      <c r="D95" s="72" t="s">
+        <v>254</v>
+      </c>
+      <c r="G95">
+        <v>3</v>
+      </c>
+      <c r="H95">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="C39:C41"/>
     <mergeCell ref="C29:C36"/>
@@ -3121,16 +3597,19 @@
     <mergeCell ref="C50:C52"/>
     <mergeCell ref="C53:C54"/>
     <mergeCell ref="C55:C60"/>
+    <mergeCell ref="C83:C89"/>
+    <mergeCell ref="C90:C91"/>
+    <mergeCell ref="C63:C66"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="B55:B60"/>
-    <mergeCell ref="C79:C80"/>
+    <mergeCell ref="C80:C81"/>
     <mergeCell ref="C61:C62"/>
-    <mergeCell ref="C63:C65"/>
-    <mergeCell ref="C66:C68"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="C73:C75"/>
-    <mergeCell ref="C76:C78"/>
+    <mergeCell ref="C67:C69"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="C74:C76"/>
+    <mergeCell ref="C77:C79"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>